<commit_message>
Workshop-Tabelle und CVs: BMEL 2. HJ 2026 + BMLEH-Umbenennung
- Kursrunde 2. HJ 2026: die beiden englischen Durchlaeufe entfallen,
  neu Teil 2,5 (02.-03.12.2026)
- Auftraggeber ab 06.05.2025 als "Forsch.Einr. BMLEH" ausgewiesen, davor
  weiterhin BMEL (Organisationserlass des Bundeskanzlers, BGBl. 2025 Nr. 131)
- .claude/ aus den Quarto-Ressourcen ausgeschlossen und in .gitignore:
  sonst kopiert der Render die Session-Worktrees nach docs/ (52 MB)
</commit_message>
<xml_diff>
--- a/docs/CV/CVcontent.xlsx
+++ b/docs/CV/CVcontent.xlsx
@@ -1460,44 +1460,44 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>114</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -1508,10 +1508,10 @@
         <v>99</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -1522,10 +1522,10 @@
         <v>99</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -1536,80 +1536,80 @@
         <v>99</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>79</v>
+        <v>137</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>99</v>
+        <v>137</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>86</v>
+        <v>137</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>86</v>
+        <v>137</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -1620,10 +1620,10 @@
         <v>137</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -1634,10 +1634,10 @@
         <v>137</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>91</v>
+        <v>144</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>91</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1648,10 +1648,10 @@
         <v>137</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>89</v>
+        <v>138</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>89</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1662,10 +1662,10 @@
         <v>137</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1676,10 +1676,10 @@
         <v>137</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1690,10 +1690,10 @@
         <v>137</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1704,10 +1704,10 @@
         <v>137</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1718,52 +1718,52 @@
         <v>137</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>150</v>
+        <v>117</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>150</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>92</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1774,52 +1774,52 @@
         <v>148</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>145</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>146</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1830,51 +1830,9 @@
         <v>149</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D31" s="5" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1944,11 +1902,15 @@
       <c r="H2" t="s">
         <v>167</v>
       </c>
-      <c r="I2" t="s">
-        <v>168</v>
-      </c>
-      <c r="J2" t="s">
-        <v>169</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">End-to-end analytics: clarify questions, acquire and align data, build models, and present results tailored to the audience</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">End-to-end Analytics: Fragestellungen präzisieren, Daten beschaffen und vereinheitlichen, Modelle entwickeln und Ergebnisse publikumsgerecht aufbereiten</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1974,11 +1936,15 @@
       <c r="H3" t="s">
         <v>167</v>
       </c>
-      <c r="I3" t="s">
-        <v>170</v>
-      </c>
-      <c r="J3" t="s">
-        <v>171</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Building and automating reproducible analysis and reporting pipelines in R and Python (Quarto)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aufbau und Automatisierung reproduzierbarer Analyse- und Reporting-Pipelines in R und Python (Quarto)</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -2004,11 +1970,15 @@
       <c r="H4" t="s">
         <v>167</v>
       </c>
-      <c r="I4" t="s">
-        <v>172</v>
-      </c>
-      <c r="J4" t="s">
-        <v>173</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scientific reports and publications, systematic reviews and meta-analyses</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wissenschaftliche Berichte und Publikationen, Systematic Reviews und Meta-Analysen</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -2035,40 +2005,40 @@
         <v>167</v>
       </c>
       <c r="I5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>43466</v>
+        <v>46113</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="D6" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="E6" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="G6" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="H6" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="I6" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="J6" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7">
@@ -2095,10 +2065,10 @@
         <v>182</v>
       </c>
       <c r="I7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8">
@@ -2125,10 +2095,10 @@
         <v>182</v>
       </c>
       <c r="I8" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9">
@@ -2155,40 +2125,40 @@
         <v>182</v>
       </c>
       <c r="I9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>46113</v>
+        <v>43405</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="D10" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="F10" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="G10" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="H10" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="I10" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="J10" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="11">
@@ -2215,40 +2185,42 @@
         <v>196</v>
       </c>
       <c r="I11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J11" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>43405</v>
-      </c>
-      <c r="B12" s="7"/>
+        <v>42248</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>43465</v>
+      </c>
       <c r="C12" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="D12" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="E12" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="F12" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="G12" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H12" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="I12" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="J12" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13">
@@ -2277,10 +2249,10 @@
         <v>204</v>
       </c>
       <c r="I13" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14">
@@ -2309,10 +2281,10 @@
         <v>204</v>
       </c>
       <c r="I14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="J14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15">
@@ -2341,42 +2313,42 @@
         <v>204</v>
       </c>
       <c r="I15" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J15" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>42248</v>
+        <v>42005</v>
       </c>
       <c r="B16" s="7" t="n">
-        <v>43465</v>
+        <v>42246</v>
       </c>
       <c r="C16" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="D16" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="E16" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="F16" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="G16" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="H16" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="I16" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="J16" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17">
@@ -2405,41 +2377,9 @@
         <v>215</v>
       </c>
       <c r="I17" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J17" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="n">
-        <v>42005</v>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>42246</v>
-      </c>
-      <c r="C18" t="s">
-        <v>213</v>
-      </c>
-      <c r="D18" t="s">
-        <v>213</v>
-      </c>
-      <c r="E18" t="s">
-        <v>165</v>
-      </c>
-      <c r="F18" t="s">
-        <v>165</v>
-      </c>
-      <c r="G18" t="s">
-        <v>214</v>
-      </c>
-      <c r="H18" t="s">
-        <v>215</v>
-      </c>
-      <c r="I18" t="s">
-        <v>218</v>
-      </c>
-      <c r="J18" t="s">
         <v>219</v>
       </c>
     </row>

</xml_diff>